<commit_message>
feat : api connected to admin
</commit_message>
<xml_diff>
--- a/app/api/data/participants.sample.xlsx
+++ b/app/api/data/participants.sample.xlsx
@@ -1,45 +1,113 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\WCL\app\api\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EB847F2-724B-4BCB-B789-112CAB2D4287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>display_name</t>
+  </si>
+  <si>
+    <t>dob</t>
+  </si>
+  <si>
+    <t>emp102</t>
+  </si>
+  <si>
+    <t>Priya Patel</t>
+  </si>
+  <si>
+    <t>15/08/2000</t>
+  </si>
+  <si>
+    <t>emp103</t>
+  </si>
+  <si>
+    <t>Rohan Gupta</t>
+  </si>
+  <si>
+    <t>1999-11-02</t>
+  </si>
+  <si>
+    <t>emp104</t>
+  </si>
+  <si>
+    <t>Ananya Iyer</t>
+  </si>
+  <si>
+    <t>emp105</t>
+  </si>
+  <si>
+    <t>Vikram Singh</t>
+  </si>
+  <si>
+    <t>2002-01-25</t>
+  </si>
+  <si>
+    <t>emp106</t>
+  </si>
+  <si>
+    <t>Sneha Reddy</t>
+  </si>
+  <si>
+    <t>2000-06-30</t>
+  </si>
+  <si>
+    <t>emp107</t>
+  </si>
+  <si>
+    <t>Arjun Nair</t>
+  </si>
+  <si>
+    <t>1998-09-19</t>
+  </si>
+  <si>
+    <t>emp108</t>
+  </si>
+  <si>
+    <t>Kavya Menon</t>
+  </si>
+  <si>
+    <t>2001-12-07</t>
+  </si>
+  <si>
+    <t>2004-15-08</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="60" formatCode="yyyy-mm-dd"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -65,15 +133,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -398,114 +473,108 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.796875" customWidth="1"/>
+    <col min="2" max="2" width="23.5" customWidth="1"/>
+    <col min="3" max="3" width="19.19921875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>username</v>
-      </c>
-      <c r="B1" t="str">
-        <v>display_name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>dob</v>
-      </c>
-      <c r="D1" t="str">
-        <v>secret</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>emp101</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Aarav Sharma</v>
-      </c>
-      <c r="C2" s="1">
-        <v>36964.22928240741</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>emp102</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Priya Patel</v>
-      </c>
-      <c r="C3" t="str">
-        <v>15/08/2000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>emp103</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Rohan Gupta</v>
-      </c>
-      <c r="C4" t="str">
-        <v>1999-11-02</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>emp104</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Ananya Iyer</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>emp105</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Vikram Singh</v>
-      </c>
-      <c r="C6" t="str">
-        <v>2002-01-25</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Vikram@2026</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>emp106</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Sneha Reddy</v>
-      </c>
-      <c r="C7" t="str">
-        <v>2000-06-30</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>emp107</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Arjun Nair</v>
-      </c>
-      <c r="C8" t="str">
-        <v>1998-09-19</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>emp108</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Kavya Menon</v>
-      </c>
-      <c r="C9" t="str">
-        <v>2001-12-07</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+    <ignoredError sqref="A1:C1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat : data ingestion
</commit_message>
<xml_diff>
--- a/app/api/data/participants.sample.xlsx
+++ b/app/api/data/participants.sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\WCL\app\api\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EB847F2-724B-4BCB-B789-112CAB2D4287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA5492BE-30E0-4EBD-838A-83FBCCDDF2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>username</t>
   </si>
@@ -31,74 +31,191 @@
     <t>dob</t>
   </si>
   <si>
-    <t>emp102</t>
-  </si>
-  <si>
-    <t>Priya Patel</t>
-  </si>
-  <si>
-    <t>15/08/2000</t>
-  </si>
-  <si>
-    <t>emp103</t>
-  </si>
-  <si>
-    <t>Rohan Gupta</t>
-  </si>
-  <si>
-    <t>1999-11-02</t>
-  </si>
-  <si>
-    <t>emp104</t>
-  </si>
-  <si>
-    <t>Ananya Iyer</t>
-  </si>
-  <si>
-    <t>emp105</t>
-  </si>
-  <si>
-    <t>Vikram Singh</t>
-  </si>
-  <si>
-    <t>2002-01-25</t>
-  </si>
-  <si>
-    <t>emp106</t>
-  </si>
-  <si>
-    <t>Sneha Reddy</t>
-  </si>
-  <si>
-    <t>2000-06-30</t>
-  </si>
-  <si>
-    <t>emp107</t>
-  </si>
-  <si>
-    <t>Arjun Nair</t>
-  </si>
-  <si>
-    <t>1998-09-19</t>
-  </si>
-  <si>
-    <t>emp108</t>
-  </si>
-  <si>
-    <t>Kavya Menon</t>
-  </si>
-  <si>
-    <t>2001-12-07</t>
-  </si>
-  <si>
-    <t>2004-15-08</t>
+    <t>emp001</t>
+  </si>
+  <si>
+    <t>Aarav Sharma</t>
+  </si>
+  <si>
+    <t>emp002</t>
+  </si>
+  <si>
+    <t>Vivaan Verma</t>
+  </si>
+  <si>
+    <t>emp003</t>
+  </si>
+  <si>
+    <t>Aditya Patel</t>
+  </si>
+  <si>
+    <t>emp004</t>
+  </si>
+  <si>
+    <t>Arjun Gupta</t>
+  </si>
+  <si>
+    <t>emp005</t>
+  </si>
+  <si>
+    <t>Krishna Joshi</t>
+  </si>
+  <si>
+    <t>emp006</t>
+  </si>
+  <si>
+    <t>Siddharth Kulkarni</t>
+  </si>
+  <si>
+    <t>emp007</t>
+  </si>
+  <si>
+    <t>Karan Reddy</t>
+  </si>
+  <si>
+    <t>emp008</t>
+  </si>
+  <si>
+    <t>Harsh Nair</t>
+  </si>
+  <si>
+    <t>emp009</t>
+  </si>
+  <si>
+    <t>Yash Rao</t>
+  </si>
+  <si>
+    <t>emp010</t>
+  </si>
+  <si>
+    <t>Nikhil Singh</t>
+  </si>
+  <si>
+    <t>emp011</t>
+  </si>
+  <si>
+    <t>Rohan Mehta</t>
+  </si>
+  <si>
+    <t>emp012</t>
+  </si>
+  <si>
+    <t>Rahul Agarwal</t>
+  </si>
+  <si>
+    <t>emp013</t>
+  </si>
+  <si>
+    <t>Aman Chawla</t>
+  </si>
+  <si>
+    <t>emp014</t>
+  </si>
+  <si>
+    <t>Akash Desai</t>
+  </si>
+  <si>
+    <t>emp015</t>
+  </si>
+  <si>
+    <t>Ritik Patil</t>
+  </si>
+  <si>
+    <t>emp016</t>
+  </si>
+  <si>
+    <t>Ananya Mishra</t>
+  </si>
+  <si>
+    <t>emp017</t>
+  </si>
+  <si>
+    <t>Aditi Arora</t>
+  </si>
+  <si>
+    <t>emp018</t>
+  </si>
+  <si>
+    <t>Sneha Khanna</t>
+  </si>
+  <si>
+    <t>emp019</t>
+  </si>
+  <si>
+    <t>Pooja Bhat</t>
+  </si>
+  <si>
+    <t>emp020</t>
+  </si>
+  <si>
+    <t>Neha Vyas</t>
+  </si>
+  <si>
+    <t>emp021</t>
+  </si>
+  <si>
+    <t>Kavya Sharma</t>
+  </si>
+  <si>
+    <t>emp022</t>
+  </si>
+  <si>
+    <t>Meera Verma</t>
+  </si>
+  <si>
+    <t>emp023</t>
+  </si>
+  <si>
+    <t>Riya Patel</t>
+  </si>
+  <si>
+    <t>emp024</t>
+  </si>
+  <si>
+    <t>Ishita Gupta</t>
+  </si>
+  <si>
+    <t>emp025</t>
+  </si>
+  <si>
+    <t>Anjali Joshi</t>
+  </si>
+  <si>
+    <t>emp026</t>
+  </si>
+  <si>
+    <t>Nandini Kulkarni</t>
+  </si>
+  <si>
+    <t>emp027</t>
+  </si>
+  <si>
+    <t>Shruti Reddy</t>
+  </si>
+  <si>
+    <t>emp028</t>
+  </si>
+  <si>
+    <t>Tanvi Nair</t>
+  </si>
+  <si>
+    <t>emp029</t>
+  </si>
+  <si>
+    <t>Muskan Rao</t>
+  </si>
+  <si>
+    <t>emp030</t>
+  </si>
+  <si>
+    <t>Diya Singh</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -108,6 +225,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -133,8 +257,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -474,12 +601,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.796875" customWidth="1"/>
     <col min="2" max="2" width="23.5" customWidth="1"/>
-    <col min="3" max="3" width="19.19921875" customWidth="1"/>
+    <col min="3" max="3" width="19.19921875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -489,90 +616,344 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3">
+        <v>38666</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" s="3">
+        <v>36167</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C4" s="3">
+        <v>37207</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" s="3">
+        <v>37940</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3">
+        <v>38425</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="3">
+        <v>35855</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="3">
+        <v>35969</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3">
+        <v>38635</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="3">
+        <v>36388</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="3">
+        <v>36639</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" t="s">
-        <v>22</v>
+      <c r="B12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="3">
+        <v>36216</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="3">
+        <v>36786</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="3">
+        <v>36244</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="3">
+        <v>37190</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="3">
+        <v>36233</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="3">
+        <v>38329</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="3">
+        <v>37160</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="3">
+        <v>36300</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="3">
+        <v>37267</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="3">
+        <v>37172</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="3">
+        <v>37577</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="3">
+        <v>38408</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="3">
+        <v>37005</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="3">
+        <v>38632</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="3">
+        <v>38542</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="3">
+        <v>37033</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="3">
+        <v>37496</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="3">
+        <v>37073</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="3">
+        <v>38365</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" s="3">
+        <v>37419</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A1:C1" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>